<commit_message>
Revised the final paper rubric and coding leader set up
</commit_message>
<xml_diff>
--- a/Group, Coding Assignment, Leading Discussion/Group, Coding Assignment, Leading Discussion.xlsx
+++ b/Group, Coding Assignment, Leading Discussion/Group, Coding Assignment, Leading Discussion.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jared_Edgerton\Dropbox\teaching_material\PSU\soda_501\Group, Coding Assignment, Leading Discussion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4DF6A56-D79C-487D-820B-41FF27C0A9F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9344EF4-C5DB-4F2F-BF6F-2F9D2623A2F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{EC1FA02E-612C-494A-963C-FE1C97348D14}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{EC1FA02E-612C-494A-963C-FE1C97348D14}"/>
   </bookViews>
   <sheets>
     <sheet name="Group" sheetId="1" r:id="rId1"/>
@@ -461,9 +461,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7DA3E93E-82E4-4A88-9248-09907879C205}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -471,7 +471,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -479,7 +479,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -487,7 +487,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -495,7 +495,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -511,9 +511,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F1E65C7-7609-49DC-884A-77D4B1C17F42}">
   <dimension ref="A1:B15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -521,12 +521,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -534,12 +534,12 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -547,7 +547,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -555,7 +555,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -563,7 +563,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -571,25 +571,22 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
-      <c r="B10" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -597,7 +594,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -605,13 +602,16 @@
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
         <v>14</v>
       </c>
     </row>
@@ -623,9 +623,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70ED5127-DBB8-4B1E-8DA2-EFF09F108950}">
   <dimension ref="A1:B15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -633,12 +633,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -646,7 +646,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -654,7 +654,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -662,12 +662,12 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -675,7 +675,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -683,12 +683,12 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -696,17 +696,17 @@
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -714,7 +714,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -722,7 +722,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>

</xml_diff>